<commit_message>
docs(samples): add full-page PDF, Word and Excel samples and a richer glossary
Care instructions (PDF), warranty terms (Word, A4) and a spare parts list (Excel), one page
each. The glossary sample holds terms of the German PDF and one row for each import rule.
</commit_message>
<xml_diff>
--- a/samples/glossar_beispiel.xlsx
+++ b/samples/glossar_beispiel.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,46 +417,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>en</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>de_synonyme</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>en_synonyme</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>beschreibung</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>nicht_uebersetzen</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>kategorie</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -461,30 +475,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kochinsel</t>
+          <t>Arbeitsplatte</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>cooking island</t>
+          <t>worktop</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Insel</t>
+          <t>Küchenarbeitsplatte</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>kitchen island</t>
+          <t>countertop</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Freistehender Küchenblock</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>Arbeitsfläche über den Unterschränken</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>technical</t>
@@ -499,22 +512,29 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Zargenprofil</t>
+          <t>Frontblende</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>frame profile</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+          <t>door front</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Front; Blende</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>front</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Rahmenprofil für Glastüren</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>Sichtbare Vorderseite von Tür oder Schublade</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>technical</t>
@@ -529,28 +549,293 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ProLine X</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+          <t>beschichtete Spanplatte</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>melamine-faced chipboard</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>melaminbeschichtete Spanplatte</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Produktname</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
+          <t>Plattenwerkstoff des Korpus</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dübel</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>wall plug</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Wanddübel</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Befestigungsmittel für die Wandmontage</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Scharnier</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>hinge</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Möbelscharnier</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Küchenfachberater</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>kitchen design consultant</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Küchenberater</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Ansprechpartner im Fachhandel</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Mehrwertsteuer</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MwSt.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>value added tax</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HS-9001</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Artikelnummer Hängeschrank, bleibt unverändert</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>product</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sockelblende</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>plinth</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Sockel</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>kickboard</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Blende unter den Unterschränken</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Glastür</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>glass door</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Unbekannte Kategorie und Status: technical / approved</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>irgendwas</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>unbekannt</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Seitenwand</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Übersetzung fehlt: wird übersprungen</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Arbeitsplatte</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>work surface</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Zweites Mal in der Datei: wird übersprungen</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>approved</t>
         </is>

</xml_diff>